<commit_message>
Updated Python File Excel File
</commit_message>
<xml_diff>
--- a/CAP776.xlsx
+++ b/CAP776.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="82">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -271,6 +271,9 @@
   </si>
   <si>
     <t>Prepare for the CA.</t>
+  </si>
+  <si>
+    <t>Prepare for the CA</t>
   </si>
 </sst>
 </file>
@@ -2786,26 +2789,50 @@
       </c>
     </row>
     <row r="30" spans="1:14">
-      <c r="A30" s="8"/>
-      <c r="B30" s="9"/>
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
-      <c r="G30" s="9"/>
-      <c r="H30" s="9"/>
-      <c r="I30" s="13" t="str">
+      <c r="A30" s="8">
+        <v>46271</v>
+      </c>
+      <c r="B30" s="9">
+        <v>360</v>
+      </c>
+      <c r="C30" s="9">
+        <v>60</v>
+      </c>
+      <c r="D30" s="9">
+        <v>120</v>
+      </c>
+      <c r="E30" s="9">
+        <v>0</v>
+      </c>
+      <c r="F30" s="9">
+        <v>150</v>
+      </c>
+      <c r="G30" s="9">
+        <v>3</v>
+      </c>
+      <c r="H30" s="9">
+        <v>120</v>
+      </c>
+      <c r="I30" s="13">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J30" s="13" t="str">
+        <v>810</v>
+      </c>
+      <c r="J30" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K30" s="14"/>
-      <c r="L30" s="14"/>
-      <c r="M30" s="14"/>
-      <c r="N30" s="16"/>
+        <v>630</v>
+      </c>
+      <c r="K30" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="L30" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="M30" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="N30" s="16" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="31" spans="1:14">
       <c r="A31" s="8"/>

</xml_diff>